<commit_message>
last changes before ordering
</commit_message>
<xml_diff>
--- a/Strommessplatine/Project Outputs for Strommessplatine/Rev02/BOM/BOM_Strommessplatine_Default_Rev02.xlsx
+++ b/Strommessplatine/Project Outputs for Strommessplatine/Rev02/BOM/BOM_Strommessplatine_Default_Rev02.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ilhan\Documents\uz_per_external_current_sensing\Strommessplatine\Project Outputs for Strommessplatine\Rev02\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{265A9E7F-1B36-4CC6-B1AB-D1AEC7C74DA2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{645E6036-DA3C-45B4-BA59-2B6AEEFDC8D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1837" yWindow="1837" windowWidth="16201" windowHeight="9308" xr2:uid="{B663A356-AF10-4E9C-A631-20B5C5521A82}"/>
+    <workbookView xWindow="735" yWindow="735" windowWidth="16200" windowHeight="9308" xr2:uid="{5A040E24-5792-48E7-BCE9-ED5EBB844B36}"/>
   </bookViews>
   <sheets>
     <sheet name="BOM_Strommessplatine_Default_Re" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="167" uniqueCount="135">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="167" uniqueCount="136">
   <si>
     <t>Name</t>
   </si>
@@ -95,13 +95,13 @@
     <t>C14663</t>
   </si>
   <si>
-    <t>27nF</t>
+    <t>27 nF</t>
   </si>
   <si>
     <t>C6</t>
   </si>
   <si>
-    <t>C162433</t>
+    <t>C519543</t>
   </si>
   <si>
     <t>1 µF</t>
@@ -227,13 +227,16 @@
     <t>C475110</t>
   </si>
   <si>
+    <t>R-RJ45R10P-B000</t>
+  </si>
+  <si>
+    <t>J3</t>
+  </si>
+  <si>
     <t>615008142621</t>
   </si>
   <si>
-    <t>J3</t>
-  </si>
-  <si>
-    <t>C5157943</t>
+    <t>C386758</t>
   </si>
   <si>
     <t>IPL1-102-02-L-D-K</t>
@@ -413,7 +416,7 @@
     <t>CASR X-NP</t>
   </si>
   <si>
-    <t>ADA4940-1ARZ</t>
+    <t>THS4521</t>
   </si>
   <si>
     <t>U4A, U4B, U4C, U4D</t>
@@ -422,7 +425,7 @@
     <t>ADA4940-1ARZ-R7</t>
   </si>
   <si>
-    <t>C459899</t>
+    <t>C16092</t>
   </si>
   <si>
     <t>TPS7A49</t>
@@ -839,7 +842,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7150DEF7-C588-4639-A648-DE8BCB9B0DE7}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2EAAACC6-D99C-48ED-8FB6-A9A6C2539C8A}">
   <dimension ref="A1:D42"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
@@ -927,7 +930,7 @@
         <v>19</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="D6" s="2" t="s">
         <v>20</v>
@@ -1137,302 +1140,302 @@
         <v>63</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="D21" s="2" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A22" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A23" s="2" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="D23" s="2" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A24" s="2" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="D24" s="2" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A25" s="2" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="D25" s="2" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A26" s="2" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="D26" s="2" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A27" s="2" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="D27" s="2" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A28" s="2" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="D28" s="2" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A29" s="2" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="D29" s="2" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A30" s="2" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="C30" s="2" t="s">
         <v>23</v>
       </c>
       <c r="D30" s="2" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A31" s="2" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="C31" s="2" t="s">
         <v>23</v>
       </c>
       <c r="D31" s="2" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A32" s="2" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="C32" s="2" t="s">
         <v>23</v>
       </c>
       <c r="D32" s="2" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A33" s="2" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="D33" s="2" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A34" s="2" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="D34" s="2" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A35" s="2" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="B35" s="2" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="D35" s="2" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A36" s="2" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="D36" s="2" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A37" s="2" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="C37" s="2" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="D37" s="2" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A38" s="2" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="B38" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="C38" s="2" t="s">
         <v>119</v>
       </c>
-      <c r="C38" s="2" t="s">
-        <v>118</v>
-      </c>
       <c r="D38" s="2" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A39" s="2" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="C39" s="2" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="D39" s="1"/>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A40" s="2" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="B40" s="2" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="C40" s="2" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="D40" s="2" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A41" s="2" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="B41" s="2" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="C41" s="2" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="D41" s="2" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A42" s="2" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="B42" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="C42" s="2" t="s">
         <v>133</v>
       </c>
-      <c r="C42" s="2" t="s">
-        <v>132</v>
-      </c>
       <c r="D42" s="2" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
to do: RJ45 L2 Thermal relief
</commit_message>
<xml_diff>
--- a/Strommessplatine/Project Outputs for Strommessplatine/Rev02/BOM/BOM_Strommessplatine_Default_Rev02.xlsx
+++ b/Strommessplatine/Project Outputs for Strommessplatine/Rev02/BOM/BOM_Strommessplatine_Default_Rev02.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ilhan\Documents\uz_per_external_current_sensing\Strommessplatine\Project Outputs for Strommessplatine\Rev02\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{645E6036-DA3C-45B4-BA59-2B6AEEFDC8D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{6BE50360-54AA-4D3A-9914-76A78CBF4366}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="735" yWindow="735" windowWidth="16200" windowHeight="9308" xr2:uid="{5A040E24-5792-48E7-BCE9-ED5EBB844B36}"/>
+    <workbookView xWindow="735" yWindow="735" windowWidth="16200" windowHeight="9308" xr2:uid="{6045F6E9-BE13-462B-AA61-7D692C785587}"/>
   </bookViews>
   <sheets>
     <sheet name="BOM_Strommessplatine_Default_Re" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="167" uniqueCount="136">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="163" uniqueCount="135">
   <si>
     <t>Name</t>
   </si>
@@ -77,7 +77,7 @@
     <t>10µF</t>
   </si>
   <si>
-    <t>C3, C4, C8, C9, C56, C60, C62</t>
+    <t>C3, C4, C8, C9, C14, C56, C60, C62</t>
   </si>
   <si>
     <t>C_1206</t>
@@ -114,9 +114,6 @@
   </si>
   <si>
     <t>C309479</t>
-  </si>
-  <si>
-    <t>C14</t>
   </si>
   <si>
     <t>C15</t>
@@ -842,8 +839,8 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2EAAACC6-D99C-48ED-8FB6-A9A6C2539C8A}">
-  <dimension ref="A1:D42"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{048C3E1C-39FC-4192-A2F6-83CCDE92C0DB}">
+  <dimension ref="A1:D41"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="17.9296875" customWidth="1"/>
@@ -952,27 +949,27 @@
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A8" s="2" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="B8" s="2" t="s">
         <v>25</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A9" s="2" t="s">
-        <v>15</v>
+        <v>26</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>6</v>
+        <v>23</v>
       </c>
       <c r="D9" s="2" t="s">
         <v>17</v>
@@ -980,462 +977,448 @@
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A10" s="2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>23</v>
+        <v>30</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>17</v>
+        <v>31</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A11" s="2" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>31</v>
+        <v>23</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A12" s="2" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="C12" s="2" t="s">
         <v>23</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A13" s="2" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="C13" s="2" t="s">
         <v>23</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A14" s="2" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>23</v>
+        <v>43</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A15" s="2" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A16" s="2" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="B16" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="C16" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="C16" s="2" t="s">
-        <v>48</v>
-      </c>
       <c r="D16" s="2" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A17" s="2" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A18" s="2" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>48</v>
+        <v>55</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A19" s="2" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A20" s="2" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A21" s="2" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="D21" s="2" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A22" s="2" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A23" s="2" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="D23" s="2" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A24" s="2" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="D24" s="2" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A25" s="2" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="B25" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="C25" s="2" t="s">
         <v>79</v>
       </c>
-      <c r="C25" s="2" t="s">
-        <v>80</v>
-      </c>
       <c r="D25" s="2" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A26" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="D26" s="2" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A27" s="2" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="D27" s="2" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A28" s="2" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="D28" s="2" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A29" s="2" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>80</v>
+        <v>23</v>
       </c>
       <c r="D29" s="2" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A30" s="2" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="C30" s="2" t="s">
         <v>23</v>
       </c>
       <c r="D30" s="2" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A31" s="2" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="C31" s="2" t="s">
         <v>23</v>
       </c>
       <c r="D31" s="2" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A32" s="2" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>23</v>
+        <v>79</v>
       </c>
       <c r="D32" s="2" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A33" s="2" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="D33" s="2" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A34" s="2" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="D34" s="2" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A35" s="2" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="B35" s="2" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="D35" s="2" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A36" s="2" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>80</v>
+        <v>116</v>
       </c>
       <c r="D36" s="2" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A37" s="2" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="C37" s="2" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="D37" s="2" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A38" s="2" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="C38" s="2" t="s">
-        <v>119</v>
-      </c>
-      <c r="D38" s="2" t="s">
-        <v>121</v>
-      </c>
+        <v>123</v>
+      </c>
+      <c r="D38" s="1"/>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A39" s="2" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="C39" s="2" t="s">
-        <v>124</v>
-      </c>
-      <c r="D39" s="1"/>
+        <v>126</v>
+      </c>
+      <c r="D39" s="2" t="s">
+        <v>127</v>
+      </c>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A40" s="2" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="B40" s="2" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
       <c r="C40" s="2" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="D40" s="2" t="s">
-        <v>128</v>
+        <v>131</v>
       </c>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A41" s="2" t="s">
-        <v>129</v>
+        <v>132</v>
       </c>
       <c r="B41" s="2" t="s">
-        <v>130</v>
+        <v>133</v>
       </c>
       <c r="C41" s="2" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="D41" s="2" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A42" s="2" t="s">
-        <v>133</v>
-      </c>
-      <c r="B42" s="2" t="s">
         <v>134</v>
-      </c>
-      <c r="C42" s="2" t="s">
-        <v>133</v>
-      </c>
-      <c r="D42" s="2" t="s">
-        <v>135</v>
       </c>
     </row>
   </sheetData>

</xml_diff>